<commit_message>
v1.2: descuentos sobre el total liquidado, signos +/-, ficha individual, envio por correo y documentacion
</commit_message>
<xml_diff>
--- a/ejemplos/nomina_marzo_2026.xlsx
+++ b/ejemplos/nomina_marzo_2026.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M10"/>
+  <dimension ref="A1:N10"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -412,6 +412,7 @@
     <col min="11" max="11" width="10.83203125" customWidth="1"/>
     <col min="12" max="12" width="18.83203125" customWidth="1"/>
     <col min="13" max="13" width="15.83203125" customWidth="1"/>
+    <col min="14" max="14" width="26.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -454,6 +455,9 @@
       <c r="M1" t="str">
         <v>Otros descuentos</v>
       </c>
+      <c r="N1" t="str">
+        <v>Correo</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -495,6 +499,9 @@
       <c r="M2">
         <v>0</v>
       </c>
+      <c r="N2" t="str">
+        <v>ana.perez@banco.com.co</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -536,6 +543,9 @@
       <c r="M3">
         <v>0</v>
       </c>
+      <c r="N3" t="str">
+        <v>carlos.gomez@banco.com.co</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -577,6 +587,9 @@
       <c r="M4">
         <v>50000</v>
       </c>
+      <c r="N4" t="str">
+        <v>marta.ruiz@banco.com.co</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -618,6 +631,9 @@
       <c r="M5">
         <v>0</v>
       </c>
+      <c r="N5" t="str">
+        <v>jorge.castro@banco.com.co</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -659,6 +675,9 @@
       <c r="M6">
         <v>0</v>
       </c>
+      <c r="N6" t="str">
+        <v>ejemplo@banco.com.co</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -700,6 +719,9 @@
       <c r="M7">
         <v>0</v>
       </c>
+      <c r="N7" t="str">
+        <v>diana.ortiz@banco.com.co</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -741,6 +763,9 @@
       <c r="M8">
         <v>0</v>
       </c>
+      <c r="N8" t="str">
+        <v>pedro.sanchez@banco.com.co</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -782,6 +807,9 @@
       <c r="M9">
         <v>0</v>
       </c>
+      <c r="N9" t="str">
+        <v>laura.mejia@banco.com.co</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
@@ -823,10 +851,13 @@
       <c r="M10">
         <v>0</v>
       </c>
+      <c r="N10" t="str">
+        <v>sin.cedula@banco.com.co</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N10"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>